<commit_message>
revised Stype3 Smooth linear start 2034
</commit_message>
<xml_diff>
--- a/SType3.xlsx
+++ b/SType3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/RegEco-PADAGIMO-SOLUSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{8352FCB5-3818-471B-95EA-A95253910025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85DC404A-7E4C-4BB1-8BD9-FC201651F405}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{8352FCB5-3818-471B-95EA-A95253910025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56F26C9E-5709-4ECA-B093-F76370F06E4D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BCA274C9-EF1D-4263-A604-C30810D98A49}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BCA274C9-EF1D-4263-A604-C30810D98A49}"/>
   </bookViews>
   <sheets>
     <sheet name="SType3" sheetId="1" r:id="rId1"/>
@@ -890,34 +890,34 @@
         <v>0.2</v>
       </c>
       <c r="M2">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N2">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O2">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P2">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q2">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R2">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S2">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T2">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U2">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V2">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W2">
         <v>0.9</v>
@@ -961,34 +961,34 @@
         <v>0.2</v>
       </c>
       <c r="M3">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N3">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O3">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P3">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q3">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R3">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S3">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T3">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U3">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V3">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W3">
         <v>0.9</v>
@@ -1032,34 +1032,34 @@
         <v>0.2</v>
       </c>
       <c r="M4">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N4">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O4">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P4">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q4">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R4">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S4">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T4">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U4">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V4">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W4">
         <v>0.9</v>
@@ -1103,34 +1103,34 @@
         <v>0.2</v>
       </c>
       <c r="M5">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N5">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O5">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P5">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q5">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R5">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S5">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T5">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U5">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V5">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W5">
         <v>0.9</v>
@@ -1174,34 +1174,34 @@
         <v>0.2</v>
       </c>
       <c r="M6">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N6">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O6">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P6">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q6">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R6">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S6">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T6">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U6">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V6">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W6">
         <v>0.9</v>
@@ -1245,34 +1245,34 @@
         <v>0.2</v>
       </c>
       <c r="M7">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N7">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O7">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P7">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q7">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R7">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S7">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T7">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U7">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V7">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W7">
         <v>0.9</v>
@@ -1316,34 +1316,34 @@
         <v>0.2</v>
       </c>
       <c r="M8">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N8">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O8">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P8">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q8">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R8">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S8">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T8">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U8">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V8">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W8">
         <v>0.9</v>
@@ -1387,34 +1387,34 @@
         <v>0.2</v>
       </c>
       <c r="M9">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N9">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O9">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P9">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q9">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R9">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S9">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T9">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U9">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V9">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W9">
         <v>0.9</v>
@@ -1458,34 +1458,34 @@
         <v>0.2</v>
       </c>
       <c r="M10">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N10">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O10">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P10">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q10">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R10">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S10">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T10">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U10">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V10">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W10">
         <v>0.9</v>
@@ -1529,34 +1529,34 @@
         <v>0.2</v>
       </c>
       <c r="M11">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N11">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O11">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P11">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q11">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R11">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S11">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T11">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U11">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V11">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W11">
         <v>0.9</v>
@@ -1600,34 +1600,34 @@
         <v>0.2</v>
       </c>
       <c r="M12">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N12">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O12">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P12">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q12">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R12">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S12">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T12">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U12">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V12">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W12">
         <v>0.9</v>
@@ -1671,34 +1671,34 @@
         <v>0.2</v>
       </c>
       <c r="M13">
-        <v>0.2</v>
+        <v>0.26363636363636367</v>
       </c>
       <c r="N13">
-        <v>0.2</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="O13">
-        <v>0.2</v>
+        <v>0.39090909090909093</v>
       </c>
       <c r="P13">
-        <v>0.2</v>
+        <v>0.45454545454545459</v>
       </c>
       <c r="Q13">
-        <v>0.5</v>
+        <v>0.51818181818181819</v>
       </c>
       <c r="R13">
-        <v>0.5</v>
+        <v>0.58181818181818179</v>
       </c>
       <c r="S13">
-        <v>0.5</v>
+        <v>0.6454545454545455</v>
       </c>
       <c r="T13">
-        <v>0.5</v>
+        <v>0.70909090909090911</v>
       </c>
       <c r="U13">
-        <v>0.5</v>
+        <v>0.77272727272727282</v>
       </c>
       <c r="V13">
-        <v>0.5</v>
+        <v>0.83636363636363642</v>
       </c>
       <c r="W13">
         <v>0.9</v>

</xml_diff>